<commit_message>
refactor(portfolio): harmonise currency in GBP, rename CA moyen client, add breakeven thresholds for Case B, add Limites section
</commit_message>
<xml_diff>
--- a/outputs/portfolio/business_case.xlsx
+++ b/outputs/portfolio/business_case.xlsx
@@ -871,7 +871,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Panier Moyen Historique du Segment</t>
+          <t>CA Moyen par Client sur la Période</t>
         </is>
       </c>
       <c r="B11" s="11" t="n">
@@ -1050,7 +1050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="134" customWidth="1" min="1" max="1"/>
@@ -1283,6 +1283,25 @@
       <c r="D14" s="5" t="inlineStr">
         <is>
           <t>£ Gain Net</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Seuil de Rentabilité (Coût Logistique min / SKU)</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>13.94120596590909</v>
+      </c>
+      <c r="C15" s="11">
+        <f>C11/C5</f>
+        <v/>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>£ / SKU / an min</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(portfolio): AOV for Case A, export_summary pipeline, aligned app/readme/slides, clean 12KB summary metrics
</commit_message>
<xml_diff>
--- a/outputs/portfolio/business_case.xlsx
+++ b/outputs/portfolio/business_case.xlsx
@@ -502,7 +502,7 @@
     <col width="51" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
@@ -593,7 +593,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Historique campagnes CRM</t>
+          <t>Hypothèse de travail à valider par A/B testing</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Merchandising / Substituts</t>
+          <t>Hypothèse de travail à valider par A/B testing</t>
         </is>
       </c>
     </row>
@@ -871,19 +871,19 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>CA Moyen par Client sur la Période</t>
+          <t>Valeur Moyenne d'une Commande</t>
         </is>
       </c>
       <c r="B11" s="11" t="n">
-        <v>1978.42</v>
+        <v>362.01</v>
       </c>
       <c r="C11" s="11">
-        <f>1978.42</f>
+        <f>362.01</f>
         <v/>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>£</t>
+          <t>£ / commande</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
         </is>
       </c>
       <c r="B14" s="11" t="n">
-        <v>117913.832</v>
+        <v>21575.796</v>
       </c>
       <c r="C14" s="11">
         <f>C13*C11</f>
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>41269.8412</v>
+        <v>7551.528599999999</v>
       </c>
       <c r="C16" s="11">
         <f>C14*C15</f>
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>39779.8412</v>
+        <v>6061.528599999999</v>
       </c>
       <c r="C17" s="14">
         <f>C16-C10</f>
@@ -1008,7 +1008,7 @@
         </is>
       </c>
       <c r="B18" s="10" t="n">
-        <v>0.002888307697195598</v>
+        <v>0.01578488360621451</v>
       </c>
       <c r="C18" s="10">
         <f>C9/(C11*C15)</f>
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="B19" s="15" t="n">
-        <v>26.69788</v>
+        <v>4.068139999999999</v>
       </c>
       <c r="C19" s="16">
         <f>C17/C10</f>

</xml_diff>